<commit_message>
M  database/seeders/ProductsSeeder.php M  database/seeders/xlsx/papapa.xlsx
</commit_message>
<xml_diff>
--- a/database/seeders/xlsx/papapa.xlsx
+++ b/database/seeders/xlsx/papapa.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="271">
   <si>
     <t>subcategory_id</t>
   </si>
@@ -92,592 +92,754 @@
     <t>Жаңа Гренни Смит алмасы</t>
   </si>
   <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/V4vcoeypDvCzPNCa5haBSM1cqulnJM1ZxYB3HmlU.webp</t>
+  </si>
+  <si>
+    <t>1 кг</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>Яблоки Американка</t>
+  </si>
+  <si>
+    <t>Американка алмасы</t>
+  </si>
+  <si>
+    <t>Свежие Яблоки Американка</t>
+  </si>
+  <si>
+    <t>Жаңа Американка алмасы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/5ExHnhULWOOkF0LmppGAqvE9rfwOmWCPuj0Rog90.webp</t>
+  </si>
+  <si>
+    <t>Яблоки Апорт</t>
+  </si>
+  <si>
+    <t>Апорт алмасы</t>
+  </si>
+  <si>
+    <t>Свежие Яблоки Апорт</t>
+  </si>
+  <si>
+    <t>Жаңа Апорт алмасы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/nFgJn4cLzkOfA7bnIDRaddM4FS6vKDe1GZPu7s46.webp</t>
+  </si>
+  <si>
+    <t>Бананы</t>
+  </si>
+  <si>
+    <t>Банан</t>
+  </si>
+  <si>
+    <t>Свежие Бананы</t>
+  </si>
+  <si>
+    <t>Жаңа Банан</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/zjXvEyXYccMDuuz2tKcTo8uNIcKaao1GsvlFpAiW.webp</t>
+  </si>
+  <si>
+    <t>Апельсины Египет</t>
+  </si>
+  <si>
+    <t>Мысыр апельсині</t>
+  </si>
+  <si>
+    <t>Свежие Апельсины Египет</t>
+  </si>
+  <si>
+    <t>Жаңа Мысыр апельсині</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/cy0algYdoBeONchp5mUqmBmvVgagTWlohqpQPxrW.webp</t>
+  </si>
+  <si>
+    <t>Апельсины Красные</t>
+  </si>
+  <si>
+    <t>Қызыл апельсин</t>
+  </si>
+  <si>
+    <t>Свежие Апельсины Красные</t>
+  </si>
+  <si>
+    <t>Жаңа Қызыл апельсин</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/SpAsQeKdRApiOh6XIxvVKDC8rmkXlQwgkEdRtEWU.webp</t>
+  </si>
+  <si>
+    <t>Апельсины Турция</t>
+  </si>
+  <si>
+    <t>Түрік апельсині</t>
+  </si>
+  <si>
+    <t>Свежие Апельсины Турция</t>
+  </si>
+  <si>
+    <t>Жаңа Түрік апельсині</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/6N7x2MM7FyRxuXRC2Yb3bn8ZaX1kXNNUTVNYUlI4.webp</t>
+  </si>
+  <si>
+    <t>Мандарины медовые</t>
+  </si>
+  <si>
+    <t>Бал мандарин</t>
+  </si>
+  <si>
+    <t>Свежие Мандарины медовые</t>
+  </si>
+  <si>
+    <t>Жаңа Бал мандарин</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/axEF4pH1zuyCbjtDr5cR9m43nFfV9wilLzrKUtMl.webp</t>
+  </si>
+  <si>
+    <t>Мандарины Турция</t>
+  </si>
+  <si>
+    <t>Түрік мандарині</t>
+  </si>
+  <si>
+    <t>Свежие Мандарины Турция</t>
+  </si>
+  <si>
+    <t>Жаңа Түрік мандарині</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/sUpyOqj1KJK9lLlUFSHMNUVTCcKtqkAwNarxbEan.webp</t>
+  </si>
+  <si>
+    <t>Мандарины с листиками</t>
+  </si>
+  <si>
+    <t>Жапырақты мандарин</t>
+  </si>
+  <si>
+    <t>Свежие Мандарины с листиками</t>
+  </si>
+  <si>
+    <t>Жаңа Жапырақты мандарин</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/BKYvO01W4SNgaEF4Oy5fm1jT4cesx2XFGOAAb1su.webp</t>
+  </si>
+  <si>
+    <t>Клубника</t>
+  </si>
+  <si>
+    <t>Құлпынай</t>
+  </si>
+  <si>
+    <t>Свежие Клубника</t>
+  </si>
+  <si>
+    <t>Жаңа Құлпынай</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/Xkq6p3SFhj2nSOcvj2EPWnva1EHJKPskrvkmDnYz.webp</t>
+  </si>
+  <si>
+    <t>Абрикос</t>
+  </si>
+  <si>
+    <t>Өрік</t>
+  </si>
+  <si>
+    <t>Свежие Абрикос</t>
+  </si>
+  <si>
+    <t>Жаңа Өрік</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/alMGvcQkJBx91Xa9Io3TrPNaapFQPzzxJqsOhvWg.webp</t>
+  </si>
+  <si>
+    <t>Виноград зеленый</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Жүзім </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Свежие Виноград </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Жаңа Жүзім </t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/LUPFi549rkqLbhb7Xkvpr5pC1QLVnKfpFYvHl1dV.webp</t>
+  </si>
+  <si>
+    <t>Персики</t>
+  </si>
+  <si>
+    <t>Шабдалы</t>
+  </si>
+  <si>
+    <t>Свежие Персики</t>
+  </si>
+  <si>
+    <t>Жаңа Шабдалы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/nuaTpSIb0YMm3VZwPjc85zRuuQwJpDJ7QECDDihw.webp</t>
+  </si>
+  <si>
+    <t>Ананас</t>
+  </si>
+  <si>
+    <t>Свежие Ананас</t>
+  </si>
+  <si>
+    <t>Жаңа Ананас</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/q6hpf2xbXmy1JY9TryjIDXmYzbjaukn0HE2jFyN5.webp</t>
+  </si>
+  <si>
+    <t>Манго</t>
+  </si>
+  <si>
+    <t>Свежие Манго</t>
+  </si>
+  <si>
+    <t>Жаңа Манго</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/k3tfHRbHLbLpyZRV1COKxKIm17S9wzsw9NZnOYh1.webp</t>
+  </si>
+  <si>
+    <t>Хурма</t>
+  </si>
+  <si>
+    <t>Свежие Хурма</t>
+  </si>
+  <si>
+    <t>Жаңа Хурма</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/7k4ZVquowOrKgafrVQvPLk2BR1tuciotirHjmHYh.webp</t>
+  </si>
+  <si>
+    <t>Киви</t>
+  </si>
+  <si>
+    <t>Свежие Киви</t>
+  </si>
+  <si>
+    <t>Жаңа Киви</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/1IDfYaFhQJVNbPqTSI1L5As2vPv2dEXHNN2IouLY.webp</t>
+  </si>
+  <si>
+    <t>Гранат</t>
+  </si>
+  <si>
+    <t>Анар</t>
+  </si>
+  <si>
+    <t>Свежие Гранат</t>
+  </si>
+  <si>
+    <t>Жаңа Анар</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/TkDUXKrOH8iSR3HoGCP6FrIVM9GcY5d6TfFMOr4E.webp</t>
+  </si>
+  <si>
+    <t>Груша лесная красавица</t>
+  </si>
+  <si>
+    <t>Орман ару алмұрт</t>
+  </si>
+  <si>
+    <t>Свежие Груша лесная красавица</t>
+  </si>
+  <si>
+    <t>Жаңа Орман ару алмұрт</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/MGIgxWRv3yjxZB4xhkCADnQyDOQOCnzZEa3GIrDr.webp</t>
+  </si>
+  <si>
+    <t>Груша конференция</t>
+  </si>
+  <si>
+    <t>Конференция алмұрт</t>
+  </si>
+  <si>
+    <t>Свежие Груша конференция</t>
+  </si>
+  <si>
+    <t>Жаңа Конференция алмұрт</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/WM4eTxfTst36GkFRjeWIQDdCDV0OT1WxlG7j4WhQ.webp</t>
+  </si>
+  <si>
+    <t>Лимон</t>
+  </si>
+  <si>
+    <t>Свежие Лимон</t>
+  </si>
+  <si>
+    <t>Жаңа Лимон</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/hRngaEzgwJEQCCsJuVoAauZ0P430KSn5fjzwVLFg.webp</t>
+  </si>
+  <si>
+    <t>Помело красный</t>
+  </si>
+  <si>
+    <t>Қызыл помело</t>
+  </si>
+  <si>
+    <t>Свежие Помело красный</t>
+  </si>
+  <si>
+    <t>Жаңа Қызыл помело</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/Zyv57yOOqY0cmFId6cetsClKMnkuyuIoZJHf949w.webp</t>
+  </si>
+  <si>
+    <t>Грейпфрут</t>
+  </si>
+  <si>
+    <t>Свежие Грейпфрут</t>
+  </si>
+  <si>
+    <t>Жаңа Грейпфрут</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/D6bMN3ovVFhEITSV7HjHei0hfsfKW1jzxRE9qd2v.webp</t>
+  </si>
+  <si>
+    <t>Картофель (Павлодар)</t>
+  </si>
+  <si>
+    <t>Павлодар картобы</t>
+  </si>
+  <si>
+    <t>Свежие Картофель (Павлодар)</t>
+  </si>
+  <si>
+    <t>Жаңа Павлодар картобы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/8BdYqDWYZoo4G2sTOe3yQhO75xSDRYX7iles71ZG.webp</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Морковь</t>
+  </si>
+  <si>
+    <t>Сәбіз</t>
+  </si>
+  <si>
+    <t>Свежие Морковь</t>
+  </si>
+  <si>
+    <t>Жаңа Сәбіз</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/TWyl2sNRFC1YAzKYsa7QNFRnY357LlrRRgFOZFlh.webp</t>
+  </si>
+  <si>
+    <t>Лук репчатый</t>
+  </si>
+  <si>
+    <t>Пияз</t>
+  </si>
+  <si>
+    <t>Свежие Лук репчатый</t>
+  </si>
+  <si>
+    <t>Жаңа Пияз</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/pDwPtQLUUZ0GzcZ8OGess0RjiF2mP1zuBOojyE2G.webp</t>
+  </si>
+  <si>
+    <t>Помидор</t>
+  </si>
+  <si>
+    <t>Қызанақ</t>
+  </si>
+  <si>
+    <t>Свежие Помидор</t>
+  </si>
+  <si>
+    <t>Жаңа Қызанақ</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/eTWXK7i6IgmPSvmRtS6IJ4Q8ZthzWNOOxVOAR56r.webp</t>
+  </si>
+  <si>
+    <t>Помидор розовый</t>
+  </si>
+  <si>
+    <t>Қызғылт қызанақ</t>
+  </si>
+  <si>
+    <t>Свежие Помидор розовый</t>
+  </si>
+  <si>
+    <t>Жаңа Қызғылт қызанақ</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/mFjYKomqvlK5yk8IJCH68CFN3P9YVqHPxDDj5T3v.webp</t>
+  </si>
+  <si>
+    <t>Огурцы рава</t>
+  </si>
+  <si>
+    <t>Рава қияры</t>
+  </si>
+  <si>
+    <t>Свежие Огурцы рава</t>
+  </si>
+  <si>
+    <t>Жаңа Рава қияры</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/Sy8fOJDX5fel752VHI3ng0EacBxaB8tpw0JnMoUL.webp</t>
+  </si>
+  <si>
+    <t>Огурцы миринда</t>
+  </si>
+  <si>
+    <t>Миринда қияры</t>
+  </si>
+  <si>
+    <t>Свежие Огурцы миринда</t>
+  </si>
+  <si>
+    <t>Жаңа Миринда қияры</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/0IbOYNs8vEEmXJP3VbZB6ILivzT3lnOzZfxt2zaH.webp</t>
+  </si>
+  <si>
+    <t>Капуста белокочанная</t>
+  </si>
+  <si>
+    <t>Ақ қауданды қырыққабат</t>
+  </si>
+  <si>
+    <t>Свежие Капуста белокочанная</t>
+  </si>
+  <si>
+    <t>Жаңа Ақ қауданды қырыққабат</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/eev245OHoK8yWAW9VoGqcEfVWo0aV3lL812FWpve.webp</t>
+  </si>
+  <si>
+    <t>Капуста пекинская</t>
+  </si>
+  <si>
+    <t>Пекин қырыққабаты</t>
+  </si>
+  <si>
+    <t>Свежие Капуста пекинская</t>
+  </si>
+  <si>
+    <t>Жаңа Пекин қырыққабаты</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/2klBDZBK5JOwQ15JLHO2ne9hrjLzYCuEU1RDWui7.webp</t>
+  </si>
+  <si>
+    <t>Капуста цветная</t>
+  </si>
+  <si>
+    <t>Түсті қырыққабат</t>
+  </si>
+  <si>
+    <t>Свежие Капуста цветная</t>
+  </si>
+  <si>
+    <t>Жаңа Түсті қырыққабат</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/9mi2ofmLls4Lk9Oy8UtXMc5DiVMrZcR7GGiXxSvN.webp</t>
+  </si>
+  <si>
+    <t>Брокколи</t>
+  </si>
+  <si>
+    <t>Свежие Брокколи</t>
+  </si>
+  <si>
+    <t>Жаңа Брокколи</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/6g8Ciz7dBUktouc74uFr2OhCRa8uDMjQ7WuNNoF9.webp</t>
+  </si>
+  <si>
+    <t>Баклажаны</t>
+  </si>
+  <si>
+    <t>Баклажан</t>
+  </si>
+  <si>
+    <t>Свежие Баклажаны</t>
+  </si>
+  <si>
+    <t>Жаңа Баклажан</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/NQHmWnkb7T3d7Pev1ssBzju72RxTeKtSip63olZy.webp</t>
+  </si>
+  <si>
+    <t>Свекла</t>
+  </si>
+  <si>
+    <t>Қызылша</t>
+  </si>
+  <si>
+    <t>Свежие Свекла</t>
+  </si>
+  <si>
+    <t>Жаңа Қызылша</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/ZpCLgExEIoJF6VAP1zMoKJPsEtcEK7bZJ7pM92xw.webp</t>
+  </si>
+  <si>
+    <t>Тыква</t>
+  </si>
+  <si>
+    <t>Асқабақ</t>
+  </si>
+  <si>
+    <t>Свежие Тыква</t>
+  </si>
+  <si>
+    <t>Жаңа Асқабақ</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/mOjSt27w1tRIvtQjJUY93giz6cE8DV5I1symrh69.webp</t>
+  </si>
+  <si>
+    <t>Перец светофор красный</t>
+  </si>
+  <si>
+    <t>Қызыл болгар бұрышы</t>
+  </si>
+  <si>
+    <t>Свежие Перец светофор красный</t>
+  </si>
+  <si>
+    <t>Жаңа Қызыл болгар бұрышы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/h0mSN5rLKsOQBFXrm8jFt2vWjb9QbHygi9BMxYDE.webp</t>
+  </si>
+  <si>
+    <t>Перец светофор зеленый</t>
+  </si>
+  <si>
+    <t>Жасыл болгар бұрышы</t>
+  </si>
+  <si>
+    <t>Свежие Перец светофор зеленый</t>
+  </si>
+  <si>
+    <t>Жаңа Жасыл болгар бұрышы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/iMTNvFCdFQGq1I76SOnrMZPlltIn2TcrBwgqkDFs.webp</t>
+  </si>
+  <si>
+    <t>Перец светофор желтый</t>
+  </si>
+  <si>
+    <t>Сары болгар бұрышы</t>
+  </si>
+  <si>
+    <t>Свежие Перец светофор желтый</t>
+  </si>
+  <si>
+    <t>Жаңа Сары болгар бұрышы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/kiRi7XWrB2DEZHo9kuepnYyqAqDZ3Om8gKAJhoQV.webp</t>
+  </si>
+  <si>
+    <t>Кабачки</t>
+  </si>
+  <si>
+    <t>Кабачок</t>
+  </si>
+  <si>
+    <t>Свежие Кабачки</t>
+  </si>
+  <si>
+    <t>Жаңа Кабачок</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/nx9EHVVegSeGCV4Z7RoCDnbBrlNivO45yFfw9qf2.webp</t>
+  </si>
+  <si>
+    <t>Чеснок</t>
+  </si>
+  <si>
+    <t>Сарымсақ</t>
+  </si>
+  <si>
+    <t>Свежие Чеснок</t>
+  </si>
+  <si>
+    <t>Жаңа Сарымсақ</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/swrmmmhZNtnKpTK8JuErzW1iSPQ0WV3zRcqAUZf8.webp</t>
+  </si>
+  <si>
+    <t>Перец полугорький</t>
+  </si>
+  <si>
+    <t>Жартылай ащы бұрыш</t>
+  </si>
+  <si>
+    <t>Свежие Перец полугорький</t>
+  </si>
+  <si>
+    <t>Жаңа Жартылай ащы бұрыш</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/E0mGal4qCGvUykytUjMHhAimuJCEvw2oLl0YlA7f.webp</t>
+  </si>
+  <si>
+    <t>Корень имбиря</t>
+  </si>
+  <si>
+    <t>Зімбір тамыры</t>
+  </si>
+  <si>
+    <t>Свежие Корень имбиря</t>
+  </si>
+  <si>
+    <t>Жаңа Зімбір тамыры</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/Mg6OAmjeQ0wefdMVB7Z29xAEYoeEaGPzcmrDwEFs.webp</t>
+  </si>
+  <si>
+    <t>Шампиньоны</t>
+  </si>
+  <si>
+    <t>Саңырауқұлақ шампиньон</t>
+  </si>
+  <si>
+    <t>Свежие Шампиньоны</t>
+  </si>
+  <si>
+    <t>Жаңа Саңырауқұлақ шампиньон</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/gBJQYCc76iCWfSv6Zw2UatEru2pEkVSvm3p5HZqq.webp</t>
+  </si>
+  <si>
+    <t>3.3</t>
+  </si>
+  <si>
+    <t>0.3</t>
+  </si>
+  <si>
+    <t>Вешенки</t>
+  </si>
+  <si>
+    <t>Устрица саңырауқұлағы</t>
+  </si>
+  <si>
+    <t>Свежие Вешенки</t>
+  </si>
+  <si>
+    <t>Жаңа Устрица саңырауқұлағы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/Y7J9jM5Quq8li8hAMAh0HCrOYv5kzJS3Sg65WY9f.webp</t>
+  </si>
+  <si>
+    <t>Лисички</t>
+  </si>
+  <si>
+    <t>Лисичка саңырауқұлағы</t>
+  </si>
+  <si>
+    <t>Свежие Лисички</t>
+  </si>
+  <si>
+    <t>Жаңа Лисичка саңырауқұлағы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/ZfYqxbJh0XPPICBoJ9zVIDLuk2QGeLaSjjVQBZxF.webp</t>
+  </si>
+  <si>
+    <t>Опята</t>
+  </si>
+  <si>
+    <t>Опята саңырауқұлағы</t>
+  </si>
+  <si>
+    <t>Свежие Опята</t>
+  </si>
+  <si>
+    <t>Жаңа Опята саңырауқұлағы</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/0E835RiAF1d1OBwepaYVeUA61Sncu5mXPIhxv13q.webp</t>
+  </si>
+  <si>
+    <t>Белый гриб</t>
+  </si>
+  <si>
+    <t>Ақ саңырауқұлақ</t>
+  </si>
+  <si>
+    <t>Свежие Белый гриб</t>
+  </si>
+  <si>
+    <t>Жаңа Ақ саңырауқұлақ</t>
+  </si>
+  <si>
+    <t>https://abricoz-eu.s3.eu-central-1.amazonaws.com/products/8dMeudOAT7dP9AW19N3dyX9PqngPWI1ADZjJrKc3.webp</t>
+  </si>
+  <si>
+    <t>Виноград черный</t>
+  </si>
+  <si>
+    <t>Жүзім</t>
+  </si>
+  <si>
+    <t>Свежие Виноград</t>
+  </si>
+  <si>
+    <t>Жаңа Жүзім</t>
+  </si>
+  <si>
     <t>null</t>
-  </si>
-  <si>
-    <t>1 кг</t>
-  </si>
-  <si>
-    <t>0.5</t>
-  </si>
-  <si>
-    <t>0.2</t>
-  </si>
-  <si>
-    <t>Яблоки Американка</t>
-  </si>
-  <si>
-    <t>Американка алмасы</t>
-  </si>
-  <si>
-    <t>Свежие Яблоки Американка</t>
-  </si>
-  <si>
-    <t>Жаңа Американка алмасы</t>
-  </si>
-  <si>
-    <t>Яблоки Апорт</t>
-  </si>
-  <si>
-    <t>Апорт алмасы</t>
-  </si>
-  <si>
-    <t>Свежие Яблоки Апорт</t>
-  </si>
-  <si>
-    <t>Жаңа Апорт алмасы</t>
-  </si>
-  <si>
-    <t>Бананы</t>
-  </si>
-  <si>
-    <t>Банан</t>
-  </si>
-  <si>
-    <t>Свежие Бананы</t>
-  </si>
-  <si>
-    <t>Жаңа Банан</t>
-  </si>
-  <si>
-    <t>Апельсины Египет</t>
-  </si>
-  <si>
-    <t>Мысыр апельсині</t>
-  </si>
-  <si>
-    <t>Свежие Апельсины Египет</t>
-  </si>
-  <si>
-    <t>Жаңа Мысыр апельсині</t>
-  </si>
-  <si>
-    <t>Апельсины Красные</t>
-  </si>
-  <si>
-    <t>Қызыл апельсин</t>
-  </si>
-  <si>
-    <t>Свежие Апельсины Красные</t>
-  </si>
-  <si>
-    <t>Жаңа Қызыл апельсин</t>
-  </si>
-  <si>
-    <t>Апельсины Турция</t>
-  </si>
-  <si>
-    <t>Түрік апельсині</t>
-  </si>
-  <si>
-    <t>Свежие Апельсины Турция</t>
-  </si>
-  <si>
-    <t>Жаңа Түрік апельсині</t>
-  </si>
-  <si>
-    <t>Мандарины медовые</t>
-  </si>
-  <si>
-    <t>Бал мандарин</t>
-  </si>
-  <si>
-    <t>Свежие Мандарины медовые</t>
-  </si>
-  <si>
-    <t>Жаңа Бал мандарин</t>
-  </si>
-  <si>
-    <t>Мандарины Турция</t>
-  </si>
-  <si>
-    <t>Түрік мандарині</t>
-  </si>
-  <si>
-    <t>Свежие Мандарины Турция</t>
-  </si>
-  <si>
-    <t>Жаңа Түрік мандарині</t>
-  </si>
-  <si>
-    <t>Мандарины с листиками</t>
-  </si>
-  <si>
-    <t>Жапырақты мандарин</t>
-  </si>
-  <si>
-    <t>Свежие Мандарины с листиками</t>
-  </si>
-  <si>
-    <t>Жаңа Жапырақты мандарин</t>
-  </si>
-  <si>
-    <t>Клубника</t>
-  </si>
-  <si>
-    <t>Құлпынай</t>
-  </si>
-  <si>
-    <t>Свежие Клубника</t>
-  </si>
-  <si>
-    <t>Жаңа Құлпынай</t>
-  </si>
-  <si>
-    <t>Абрикос</t>
-  </si>
-  <si>
-    <t>Өрік</t>
-  </si>
-  <si>
-    <t>Свежие Абрикос</t>
-  </si>
-  <si>
-    <t>Жаңа Өрік</t>
-  </si>
-  <si>
-    <t>Виноград (черный и зеленый Узбекистан)</t>
-  </si>
-  <si>
-    <t>Жүзім (қара және жасыл, Өзбекстан)</t>
-  </si>
-  <si>
-    <t>Свежие Виноград (черный и зеленый Узбекистан)</t>
-  </si>
-  <si>
-    <t>Жаңа Жүзім (қара және жасыл, Өзбекстан)</t>
-  </si>
-  <si>
-    <t>Персики</t>
-  </si>
-  <si>
-    <t>Шабдалы</t>
-  </si>
-  <si>
-    <t>Свежие Персики</t>
-  </si>
-  <si>
-    <t>Жаңа Шабдалы</t>
-  </si>
-  <si>
-    <t>Ананас</t>
-  </si>
-  <si>
-    <t>Свежие Ананас</t>
-  </si>
-  <si>
-    <t>Жаңа Ананас</t>
-  </si>
-  <si>
-    <t>Манго</t>
-  </si>
-  <si>
-    <t>Свежие Манго</t>
-  </si>
-  <si>
-    <t>Жаңа Манго</t>
-  </si>
-  <si>
-    <t>Хурма</t>
-  </si>
-  <si>
-    <t>Свежие Хурма</t>
-  </si>
-  <si>
-    <t>Жаңа Хурма</t>
-  </si>
-  <si>
-    <t>Киви</t>
-  </si>
-  <si>
-    <t>Свежие Киви</t>
-  </si>
-  <si>
-    <t>Жаңа Киви</t>
-  </si>
-  <si>
-    <t>Гранат</t>
-  </si>
-  <si>
-    <t>Анар</t>
-  </si>
-  <si>
-    <t>Свежие Гранат</t>
-  </si>
-  <si>
-    <t>Жаңа Анар</t>
-  </si>
-  <si>
-    <t>Груша лесная красавица</t>
-  </si>
-  <si>
-    <t>Орман ару алмұрт</t>
-  </si>
-  <si>
-    <t>Свежие Груша лесная красавица</t>
-  </si>
-  <si>
-    <t>Жаңа Орман ару алмұрт</t>
-  </si>
-  <si>
-    <t>Груша конференция</t>
-  </si>
-  <si>
-    <t>Конференция алмұрт</t>
-  </si>
-  <si>
-    <t>Свежие Груша конференция</t>
-  </si>
-  <si>
-    <t>Жаңа Конференция алмұрт</t>
-  </si>
-  <si>
-    <t>Лимон</t>
-  </si>
-  <si>
-    <t>Свежие Лимон</t>
-  </si>
-  <si>
-    <t>Жаңа Лимон</t>
-  </si>
-  <si>
-    <t>Помело красный</t>
-  </si>
-  <si>
-    <t>Қызыл помело</t>
-  </si>
-  <si>
-    <t>Свежие Помело красный</t>
-  </si>
-  <si>
-    <t>Жаңа Қызыл помело</t>
-  </si>
-  <si>
-    <t>Грейпфрут</t>
-  </si>
-  <si>
-    <t>Свежие Грейпфрут</t>
-  </si>
-  <si>
-    <t>Жаңа Грейпфрут</t>
-  </si>
-  <si>
-    <t>Картофель (Павлодар)</t>
-  </si>
-  <si>
-    <t>Павлодар картобы</t>
-  </si>
-  <si>
-    <t>Свежие Картофель (Павлодар)</t>
-  </si>
-  <si>
-    <t>Жаңа Павлодар картобы</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>Морковь</t>
-  </si>
-  <si>
-    <t>Сәбіз</t>
-  </si>
-  <si>
-    <t>Свежие Морковь</t>
-  </si>
-  <si>
-    <t>Жаңа Сәбіз</t>
-  </si>
-  <si>
-    <t>Лук репчатый</t>
-  </si>
-  <si>
-    <t>Пияз</t>
-  </si>
-  <si>
-    <t>Свежие Лук репчатый</t>
-  </si>
-  <si>
-    <t>Жаңа Пияз</t>
-  </si>
-  <si>
-    <t>Помидор</t>
-  </si>
-  <si>
-    <t>Қызанақ</t>
-  </si>
-  <si>
-    <t>Свежие Помидор</t>
-  </si>
-  <si>
-    <t>Жаңа Қызанақ</t>
-  </si>
-  <si>
-    <t>Помидор розовый</t>
-  </si>
-  <si>
-    <t>Қызғылт қызанақ</t>
-  </si>
-  <si>
-    <t>Свежие Помидор розовый</t>
-  </si>
-  <si>
-    <t>Жаңа Қызғылт қызанақ</t>
-  </si>
-  <si>
-    <t>Огурцы рава</t>
-  </si>
-  <si>
-    <t>Рава қияры</t>
-  </si>
-  <si>
-    <t>Свежие Огурцы рава</t>
-  </si>
-  <si>
-    <t>Жаңа Рава қияры</t>
-  </si>
-  <si>
-    <t>Огурцы миринда</t>
-  </si>
-  <si>
-    <t>Миринда қияры</t>
-  </si>
-  <si>
-    <t>Свежие Огурцы миринда</t>
-  </si>
-  <si>
-    <t>Жаңа Миринда қияры</t>
-  </si>
-  <si>
-    <t>Капуста белокочанная</t>
-  </si>
-  <si>
-    <t>Ақ қауданды қырыққабат</t>
-  </si>
-  <si>
-    <t>Свежие Капуста белокочанная</t>
-  </si>
-  <si>
-    <t>Жаңа Ақ қауданды қырыққабат</t>
-  </si>
-  <si>
-    <t>Капуста пекинская</t>
-  </si>
-  <si>
-    <t>Пекин қырыққабаты</t>
-  </si>
-  <si>
-    <t>Свежие Капуста пекинская</t>
-  </si>
-  <si>
-    <t>Жаңа Пекин қырыққабаты</t>
-  </si>
-  <si>
-    <t>Капуста цветная</t>
-  </si>
-  <si>
-    <t>Түсті қырыққабат</t>
-  </si>
-  <si>
-    <t>Свежие Капуста цветная</t>
-  </si>
-  <si>
-    <t>Жаңа Түсті қырыққабат</t>
-  </si>
-  <si>
-    <t>Брокколи</t>
-  </si>
-  <si>
-    <t>Свежие Брокколи</t>
-  </si>
-  <si>
-    <t>Жаңа Брокколи</t>
-  </si>
-  <si>
-    <t>Баклажаны</t>
-  </si>
-  <si>
-    <t>Баклажан</t>
-  </si>
-  <si>
-    <t>Свежие Баклажаны</t>
-  </si>
-  <si>
-    <t>Жаңа Баклажан</t>
-  </si>
-  <si>
-    <t>Свекла</t>
-  </si>
-  <si>
-    <t>Қызылша</t>
-  </si>
-  <si>
-    <t>Свежие Свекла</t>
-  </si>
-  <si>
-    <t>Жаңа Қызылша</t>
-  </si>
-  <si>
-    <t>Тыква</t>
-  </si>
-  <si>
-    <t>Асқабақ</t>
-  </si>
-  <si>
-    <t>Свежие Тыква</t>
-  </si>
-  <si>
-    <t>Жаңа Асқабақ</t>
-  </si>
-  <si>
-    <t>Перец светофор красный</t>
-  </si>
-  <si>
-    <t>Қызыл болгар бұрышы</t>
-  </si>
-  <si>
-    <t>Свежие Перец светофор красный</t>
-  </si>
-  <si>
-    <t>Жаңа Қызыл болгар бұрышы</t>
-  </si>
-  <si>
-    <t>Перец светофор зеленый</t>
-  </si>
-  <si>
-    <t>Жасыл болгар бұрышы</t>
-  </si>
-  <si>
-    <t>Свежие Перец светофор зеленый</t>
-  </si>
-  <si>
-    <t>Жаңа Жасыл болгар бұрышы</t>
-  </si>
-  <si>
-    <t>Перец светофор желтый</t>
-  </si>
-  <si>
-    <t>Сары болгар бұрышы</t>
-  </si>
-  <si>
-    <t>Свежие Перец светофор желтый</t>
-  </si>
-  <si>
-    <t>Жаңа Сары болгар бұрышы</t>
-  </si>
-  <si>
-    <t>Кабачки</t>
-  </si>
-  <si>
-    <t>Кабачок</t>
-  </si>
-  <si>
-    <t>Свежие Кабачки</t>
-  </si>
-  <si>
-    <t>Жаңа Кабачок</t>
-  </si>
-  <si>
-    <t>Чеснок</t>
-  </si>
-  <si>
-    <t>Сарымсақ</t>
-  </si>
-  <si>
-    <t>Свежие Чеснок</t>
-  </si>
-  <si>
-    <t>Жаңа Сарымсақ</t>
-  </si>
-  <si>
-    <t>Перец полугорький</t>
-  </si>
-  <si>
-    <t>Жартылай ащы бұрыш</t>
-  </si>
-  <si>
-    <t>Свежие Перец полугорький</t>
-  </si>
-  <si>
-    <t>Жаңа Жартылай ащы бұрыш</t>
-  </si>
-  <si>
-    <t>Корень имбиря</t>
-  </si>
-  <si>
-    <t>Зімбір тамыры</t>
-  </si>
-  <si>
-    <t>Свежие Корень имбиря</t>
-  </si>
-  <si>
-    <t>Жаңа Зімбір тамыры</t>
-  </si>
-  <si>
-    <t>Шампиньоны</t>
-  </si>
-  <si>
-    <t>Саңырауқұлақ шампиньон</t>
-  </si>
-  <si>
-    <t>Свежие Шампиньоны</t>
-  </si>
-  <si>
-    <t>Жаңа Саңырауқұлақ шампиньон</t>
-  </si>
-  <si>
-    <t>3.3</t>
-  </si>
-  <si>
-    <t>0.3</t>
-  </si>
-  <si>
-    <t>Вешенки</t>
-  </si>
-  <si>
-    <t>Устрица саңырауқұлағы</t>
-  </si>
-  <si>
-    <t>Свежие Вешенки</t>
-  </si>
-  <si>
-    <t>Жаңа Устрица саңырауқұлағы</t>
-  </si>
-  <si>
-    <t>Лисички</t>
-  </si>
-  <si>
-    <t>Лисичка саңырауқұлағы</t>
-  </si>
-  <si>
-    <t>Свежие Лисички</t>
-  </si>
-  <si>
-    <t>Жаңа Лисичка саңырауқұлағы</t>
-  </si>
-  <si>
-    <t>Опята</t>
-  </si>
-  <si>
-    <t>Опята саңырауқұлағы</t>
-  </si>
-  <si>
-    <t>Свежие Опята</t>
-  </si>
-  <si>
-    <t>Жаңа Опята саңырауқұлағы</t>
-  </si>
-  <si>
-    <t>Белый гриб</t>
-  </si>
-  <si>
-    <t>Ақ саңырауқұлақ</t>
-  </si>
-  <si>
-    <t>Свежие Белый гриб</t>
-  </si>
-  <si>
-    <t>Жаңа Ақ саңырауқұлақ</t>
   </si>
 </sst>
 </file>
@@ -1830,14 +1992,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="43.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="9.42857142857143" customWidth="1"/>
-    <col min="5" max="5" width="5.28571428571429" customWidth="1"/>
+    <col min="4" max="4" width="38.1428571428571" customWidth="1"/>
+    <col min="5" max="5" width="27.4285714285714" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
@@ -1968,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J3" t="s">
         <v>22</v>
@@ -2000,16 +2162,16 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G4">
         <v>1000</v>
@@ -2018,7 +2180,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="J4" t="s">
         <v>22</v>
@@ -2050,16 +2212,16 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G5">
         <v>1000</v>
@@ -2068,7 +2230,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -2100,16 +2262,16 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G6">
         <v>1000</v>
@@ -2118,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="J6" t="s">
         <v>22</v>
@@ -2150,16 +2312,16 @@
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G7">
         <v>1000</v>
@@ -2168,7 +2330,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="J7" t="s">
         <v>22</v>
@@ -2200,16 +2362,16 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G8">
         <v>1000</v>
@@ -2218,7 +2380,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="J8" t="s">
         <v>22</v>
@@ -2250,16 +2412,16 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G9">
         <v>1000</v>
@@ -2268,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="J9" t="s">
         <v>22</v>
@@ -2300,16 +2462,16 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <v>1000</v>
@@ -2318,7 +2480,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="J10" t="s">
         <v>22</v>
@@ -2350,16 +2512,16 @@
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="G11">
         <v>1000</v>
@@ -2368,7 +2530,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="J11" t="s">
         <v>22</v>
@@ -2400,16 +2562,16 @@
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="G12">
         <v>1000</v>
@@ -2418,7 +2580,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="J12" t="s">
         <v>22</v>
@@ -2450,16 +2612,16 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F13" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G13">
         <v>1000</v>
@@ -2468,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="J13" t="s">
         <v>22</v>
@@ -2500,16 +2662,16 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="G14">
         <v>1000</v>
@@ -2518,7 +2680,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="J14" t="s">
         <v>22</v>
@@ -2550,16 +2712,16 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="G15">
         <v>1000</v>
@@ -2568,7 +2730,7 @@
         <v>0</v>
       </c>
       <c r="I15" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="J15" t="s">
         <v>22</v>
@@ -2600,16 +2762,16 @@
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="G16">
         <v>1000</v>
@@ -2618,7 +2780,7 @@
         <v>0</v>
       </c>
       <c r="I16" t="s">
-        <v>21</v>
+        <v>93</v>
       </c>
       <c r="J16" t="s">
         <v>22</v>
@@ -2650,16 +2812,16 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="D17" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="G17">
         <v>1000</v>
@@ -2668,7 +2830,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="s">
-        <v>21</v>
+        <v>97</v>
       </c>
       <c r="J17" t="s">
         <v>22</v>
@@ -2700,16 +2862,16 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="E18" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="G18">
         <v>1000</v>
@@ -2718,7 +2880,7 @@
         <v>0</v>
       </c>
       <c r="I18" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="J18" t="s">
         <v>22</v>
@@ -2750,16 +2912,16 @@
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="D19" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E19" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="F19" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="G19">
         <v>1000</v>
@@ -2768,7 +2930,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="J19" t="s">
         <v>22</v>
@@ -2800,16 +2962,16 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="D20" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="G20">
         <v>1000</v>
@@ -2818,7 +2980,7 @@
         <v>0</v>
       </c>
       <c r="I20" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
       <c r="J20" t="s">
         <v>22</v>
@@ -2850,16 +3012,16 @@
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="D21" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="E21" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="F21" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="G21">
         <v>1000</v>
@@ -2868,7 +3030,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="s">
-        <v>21</v>
+        <v>115</v>
       </c>
       <c r="J21" t="s">
         <v>22</v>
@@ -2900,16 +3062,16 @@
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="E22" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="F22" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="G22">
         <v>1000</v>
@@ -2918,7 +3080,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="s">
-        <v>21</v>
+        <v>120</v>
       </c>
       <c r="J22" t="s">
         <v>22</v>
@@ -2950,16 +3112,16 @@
         <v>16</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="E23" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="F23" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="G23">
         <v>1000</v>
@@ -2968,7 +3130,7 @@
         <v>0</v>
       </c>
       <c r="I23" t="s">
-        <v>21</v>
+        <v>124</v>
       </c>
       <c r="J23" t="s">
         <v>22</v>
@@ -3000,16 +3162,16 @@
         <v>16</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="D24" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="E24" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="F24" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="G24">
         <v>1000</v>
@@ -3018,7 +3180,7 @@
         <v>0</v>
       </c>
       <c r="I24" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="J24" t="s">
         <v>22</v>
@@ -3050,16 +3212,16 @@
         <v>16</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="D25" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="E25" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="F25" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="G25">
         <v>1000</v>
@@ -3068,7 +3230,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>21</v>
+        <v>133</v>
       </c>
       <c r="J25" t="s">
         <v>22</v>
@@ -3100,16 +3262,16 @@
         <v>16</v>
       </c>
       <c r="C26" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="D26" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="E26" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="F26" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="G26">
         <v>1000</v>
@@ -3118,7 +3280,7 @@
         <v>0</v>
       </c>
       <c r="I26" t="s">
-        <v>21</v>
+        <v>138</v>
       </c>
       <c r="J26" t="s">
         <v>22</v>
@@ -3127,7 +3289,7 @@
         <v>30</v>
       </c>
       <c r="L26" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M26" t="s">
         <v>24</v>
@@ -3150,16 +3312,16 @@
         <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="D27" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="E27" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="F27" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="G27">
         <v>1000</v>
@@ -3168,7 +3330,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="s">
-        <v>21</v>
+        <v>144</v>
       </c>
       <c r="J27" t="s">
         <v>22</v>
@@ -3177,7 +3339,7 @@
         <v>30</v>
       </c>
       <c r="L27" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M27" t="s">
         <v>24</v>
@@ -3200,16 +3362,16 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="F28" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="G28">
         <v>1000</v>
@@ -3218,7 +3380,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="s">
-        <v>21</v>
+        <v>149</v>
       </c>
       <c r="J28" t="s">
         <v>22</v>
@@ -3227,7 +3389,7 @@
         <v>30</v>
       </c>
       <c r="L28" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M28" t="s">
         <v>24</v>
@@ -3250,16 +3412,16 @@
         <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
       <c r="E29" t="s">
-        <v>126</v>
+        <v>152</v>
       </c>
       <c r="F29" t="s">
-        <v>127</v>
+        <v>153</v>
       </c>
       <c r="G29">
         <v>1000</v>
@@ -3268,7 +3430,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="s">
-        <v>21</v>
+        <v>154</v>
       </c>
       <c r="J29" t="s">
         <v>22</v>
@@ -3277,7 +3439,7 @@
         <v>30</v>
       </c>
       <c r="L29" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M29" t="s">
         <v>24</v>
@@ -3300,16 +3462,16 @@
         <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>128</v>
+        <v>155</v>
       </c>
       <c r="D30" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
       <c r="E30" t="s">
-        <v>130</v>
+        <v>157</v>
       </c>
       <c r="F30" t="s">
-        <v>131</v>
+        <v>158</v>
       </c>
       <c r="G30">
         <v>1000</v>
@@ -3318,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="I30" t="s">
-        <v>21</v>
+        <v>159</v>
       </c>
       <c r="J30" t="s">
         <v>22</v>
@@ -3327,7 +3489,7 @@
         <v>30</v>
       </c>
       <c r="L30" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M30" t="s">
         <v>24</v>
@@ -3350,16 +3512,16 @@
         <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="D31" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="E31" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="F31" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="G31">
         <v>1000</v>
@@ -3368,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="I31" t="s">
-        <v>21</v>
+        <v>164</v>
       </c>
       <c r="J31" t="s">
         <v>22</v>
@@ -3377,7 +3539,7 @@
         <v>30</v>
       </c>
       <c r="L31" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M31" t="s">
         <v>24</v>
@@ -3400,16 +3562,16 @@
         <v>16</v>
       </c>
       <c r="C32" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="D32" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="E32" t="s">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="F32" t="s">
-        <v>139</v>
+        <v>168</v>
       </c>
       <c r="G32">
         <v>1000</v>
@@ -3418,7 +3580,7 @@
         <v>0</v>
       </c>
       <c r="I32" t="s">
-        <v>21</v>
+        <v>169</v>
       </c>
       <c r="J32" t="s">
         <v>22</v>
@@ -3427,7 +3589,7 @@
         <v>30</v>
       </c>
       <c r="L32" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M32" t="s">
         <v>24</v>
@@ -3450,16 +3612,16 @@
         <v>16</v>
       </c>
       <c r="C33" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="D33" t="s">
-        <v>141</v>
+        <v>171</v>
       </c>
       <c r="E33" t="s">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="F33" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="G33">
         <v>1000</v>
@@ -3468,7 +3630,7 @@
         <v>0</v>
       </c>
       <c r="I33" t="s">
-        <v>21</v>
+        <v>174</v>
       </c>
       <c r="J33" t="s">
         <v>22</v>
@@ -3477,7 +3639,7 @@
         <v>30</v>
       </c>
       <c r="L33" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M33" t="s">
         <v>24</v>
@@ -3500,16 +3662,16 @@
         <v>16</v>
       </c>
       <c r="C34" t="s">
-        <v>144</v>
+        <v>175</v>
       </c>
       <c r="D34" t="s">
-        <v>145</v>
+        <v>176</v>
       </c>
       <c r="E34" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="F34" t="s">
-        <v>147</v>
+        <v>178</v>
       </c>
       <c r="G34">
         <v>1000</v>
@@ -3518,7 +3680,7 @@
         <v>0</v>
       </c>
       <c r="I34" t="s">
-        <v>21</v>
+        <v>179</v>
       </c>
       <c r="J34" t="s">
         <v>22</v>
@@ -3527,7 +3689,7 @@
         <v>30</v>
       </c>
       <c r="L34" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M34" t="s">
         <v>24</v>
@@ -3550,16 +3712,16 @@
         <v>16</v>
       </c>
       <c r="C35" t="s">
-        <v>148</v>
+        <v>180</v>
       </c>
       <c r="D35" t="s">
-        <v>149</v>
+        <v>181</v>
       </c>
       <c r="E35" t="s">
-        <v>150</v>
+        <v>182</v>
       </c>
       <c r="F35" t="s">
-        <v>151</v>
+        <v>183</v>
       </c>
       <c r="G35">
         <v>1000</v>
@@ -3568,7 +3730,7 @@
         <v>0</v>
       </c>
       <c r="I35" t="s">
-        <v>21</v>
+        <v>184</v>
       </c>
       <c r="J35" t="s">
         <v>22</v>
@@ -3577,7 +3739,7 @@
         <v>30</v>
       </c>
       <c r="L35" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M35" t="s">
         <v>24</v>
@@ -3600,16 +3762,16 @@
         <v>16</v>
       </c>
       <c r="C36" t="s">
-        <v>152</v>
+        <v>185</v>
       </c>
       <c r="D36" t="s">
-        <v>152</v>
+        <v>185</v>
       </c>
       <c r="E36" t="s">
-        <v>153</v>
+        <v>186</v>
       </c>
       <c r="F36" t="s">
-        <v>154</v>
+        <v>187</v>
       </c>
       <c r="G36">
         <v>1000</v>
@@ -3618,7 +3780,7 @@
         <v>0</v>
       </c>
       <c r="I36" t="s">
-        <v>21</v>
+        <v>188</v>
       </c>
       <c r="J36" t="s">
         <v>22</v>
@@ -3627,7 +3789,7 @@
         <v>30</v>
       </c>
       <c r="L36" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M36" t="s">
         <v>24</v>
@@ -3650,16 +3812,16 @@
         <v>16</v>
       </c>
       <c r="C37" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="D37" t="s">
-        <v>156</v>
+        <v>190</v>
       </c>
       <c r="E37" t="s">
-        <v>157</v>
+        <v>191</v>
       </c>
       <c r="F37" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="G37">
         <v>1000</v>
@@ -3668,7 +3830,7 @@
         <v>0</v>
       </c>
       <c r="I37" t="s">
-        <v>21</v>
+        <v>193</v>
       </c>
       <c r="J37" t="s">
         <v>22</v>
@@ -3677,7 +3839,7 @@
         <v>30</v>
       </c>
       <c r="L37" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M37" t="s">
         <v>24</v>
@@ -3700,16 +3862,16 @@
         <v>16</v>
       </c>
       <c r="C38" t="s">
-        <v>159</v>
+        <v>194</v>
       </c>
       <c r="D38" t="s">
-        <v>160</v>
+        <v>195</v>
       </c>
       <c r="E38" t="s">
-        <v>161</v>
+        <v>196</v>
       </c>
       <c r="F38" t="s">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="G38">
         <v>1000</v>
@@ -3718,7 +3880,7 @@
         <v>0</v>
       </c>
       <c r="I38" t="s">
-        <v>21</v>
+        <v>198</v>
       </c>
       <c r="J38" t="s">
         <v>22</v>
@@ -3727,7 +3889,7 @@
         <v>30</v>
       </c>
       <c r="L38" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M38" t="s">
         <v>24</v>
@@ -3750,16 +3912,16 @@
         <v>16</v>
       </c>
       <c r="C39" t="s">
-        <v>163</v>
+        <v>199</v>
       </c>
       <c r="D39" t="s">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="E39" t="s">
-        <v>165</v>
+        <v>201</v>
       </c>
       <c r="F39" t="s">
-        <v>166</v>
+        <v>202</v>
       </c>
       <c r="G39">
         <v>1000</v>
@@ -3768,7 +3930,7 @@
         <v>0</v>
       </c>
       <c r="I39" t="s">
-        <v>21</v>
+        <v>203</v>
       </c>
       <c r="J39" t="s">
         <v>22</v>
@@ -3777,7 +3939,7 @@
         <v>30</v>
       </c>
       <c r="L39" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M39" t="s">
         <v>24</v>
@@ -3800,16 +3962,16 @@
         <v>16</v>
       </c>
       <c r="C40" t="s">
-        <v>167</v>
+        <v>204</v>
       </c>
       <c r="D40" t="s">
-        <v>168</v>
+        <v>205</v>
       </c>
       <c r="E40" t="s">
-        <v>169</v>
+        <v>206</v>
       </c>
       <c r="F40" t="s">
-        <v>170</v>
+        <v>207</v>
       </c>
       <c r="G40">
         <v>1000</v>
@@ -3818,7 +3980,7 @@
         <v>0</v>
       </c>
       <c r="I40" t="s">
-        <v>21</v>
+        <v>208</v>
       </c>
       <c r="J40" t="s">
         <v>22</v>
@@ -3827,7 +3989,7 @@
         <v>30</v>
       </c>
       <c r="L40" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M40" t="s">
         <v>24</v>
@@ -3850,16 +4012,16 @@
         <v>16</v>
       </c>
       <c r="C41" t="s">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="D41" t="s">
-        <v>172</v>
+        <v>210</v>
       </c>
       <c r="E41" t="s">
-        <v>173</v>
+        <v>211</v>
       </c>
       <c r="F41" t="s">
-        <v>174</v>
+        <v>212</v>
       </c>
       <c r="G41">
         <v>1000</v>
@@ -3868,7 +4030,7 @@
         <v>0</v>
       </c>
       <c r="I41" t="s">
-        <v>21</v>
+        <v>213</v>
       </c>
       <c r="J41" t="s">
         <v>22</v>
@@ -3877,7 +4039,7 @@
         <v>30</v>
       </c>
       <c r="L41" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M41" t="s">
         <v>24</v>
@@ -3900,16 +4062,16 @@
         <v>16</v>
       </c>
       <c r="C42" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="D42" t="s">
-        <v>176</v>
+        <v>215</v>
       </c>
       <c r="E42" t="s">
-        <v>177</v>
+        <v>216</v>
       </c>
       <c r="F42" t="s">
-        <v>178</v>
+        <v>217</v>
       </c>
       <c r="G42">
         <v>1000</v>
@@ -3918,7 +4080,7 @@
         <v>0</v>
       </c>
       <c r="I42" t="s">
-        <v>21</v>
+        <v>218</v>
       </c>
       <c r="J42" t="s">
         <v>22</v>
@@ -3927,7 +4089,7 @@
         <v>30</v>
       </c>
       <c r="L42" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M42" t="s">
         <v>24</v>
@@ -3950,16 +4112,16 @@
         <v>16</v>
       </c>
       <c r="C43" t="s">
-        <v>179</v>
+        <v>219</v>
       </c>
       <c r="D43" t="s">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="E43" t="s">
-        <v>181</v>
+        <v>221</v>
       </c>
       <c r="F43" t="s">
-        <v>182</v>
+        <v>222</v>
       </c>
       <c r="G43">
         <v>1000</v>
@@ -3968,7 +4130,7 @@
         <v>0</v>
       </c>
       <c r="I43" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="J43" t="s">
         <v>22</v>
@@ -3977,7 +4139,7 @@
         <v>30</v>
       </c>
       <c r="L43" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M43" t="s">
         <v>24</v>
@@ -4000,16 +4162,16 @@
         <v>16</v>
       </c>
       <c r="C44" t="s">
-        <v>183</v>
+        <v>224</v>
       </c>
       <c r="D44" t="s">
-        <v>184</v>
+        <v>225</v>
       </c>
       <c r="E44" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="F44" t="s">
-        <v>186</v>
+        <v>227</v>
       </c>
       <c r="G44">
         <v>1000</v>
@@ -4018,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="I44" t="s">
-        <v>21</v>
+        <v>228</v>
       </c>
       <c r="J44" t="s">
         <v>22</v>
@@ -4027,7 +4189,7 @@
         <v>30</v>
       </c>
       <c r="L44" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M44" t="s">
         <v>24</v>
@@ -4050,16 +4212,16 @@
         <v>16</v>
       </c>
       <c r="C45" t="s">
-        <v>187</v>
+        <v>229</v>
       </c>
       <c r="D45" t="s">
-        <v>188</v>
+        <v>230</v>
       </c>
       <c r="E45" t="s">
-        <v>189</v>
+        <v>231</v>
       </c>
       <c r="F45" t="s">
-        <v>190</v>
+        <v>232</v>
       </c>
       <c r="G45">
         <v>1000</v>
@@ -4068,7 +4230,7 @@
         <v>0</v>
       </c>
       <c r="I45" t="s">
-        <v>21</v>
+        <v>233</v>
       </c>
       <c r="J45" t="s">
         <v>22</v>
@@ -4077,7 +4239,7 @@
         <v>30</v>
       </c>
       <c r="L45" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M45" t="s">
         <v>24</v>
@@ -4100,16 +4262,16 @@
         <v>16</v>
       </c>
       <c r="C46" t="s">
-        <v>191</v>
+        <v>234</v>
       </c>
       <c r="D46" t="s">
-        <v>192</v>
+        <v>235</v>
       </c>
       <c r="E46" t="s">
-        <v>193</v>
+        <v>236</v>
       </c>
       <c r="F46" t="s">
-        <v>194</v>
+        <v>237</v>
       </c>
       <c r="G46">
         <v>1000</v>
@@ -4118,7 +4280,7 @@
         <v>0</v>
       </c>
       <c r="I46" t="s">
-        <v>21</v>
+        <v>238</v>
       </c>
       <c r="J46" t="s">
         <v>22</v>
@@ -4127,7 +4289,7 @@
         <v>30</v>
       </c>
       <c r="L46" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="M46" t="s">
         <v>24</v>
@@ -4150,16 +4312,16 @@
         <v>16</v>
       </c>
       <c r="C47" t="s">
-        <v>195</v>
+        <v>239</v>
       </c>
       <c r="D47" t="s">
-        <v>196</v>
+        <v>240</v>
       </c>
       <c r="E47" t="s">
-        <v>197</v>
+        <v>241</v>
       </c>
       <c r="F47" t="s">
-        <v>198</v>
+        <v>242</v>
       </c>
       <c r="G47">
         <v>1000</v>
@@ -4168,7 +4330,7 @@
         <v>0</v>
       </c>
       <c r="I47" t="s">
-        <v>21</v>
+        <v>243</v>
       </c>
       <c r="J47" t="s">
         <v>22</v>
@@ -4177,13 +4339,13 @@
         <v>22</v>
       </c>
       <c r="L47" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="M47" t="s">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="N47" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="O47">
         <v>1</v>
@@ -4200,16 +4362,16 @@
         <v>16</v>
       </c>
       <c r="C48" t="s">
-        <v>201</v>
+        <v>246</v>
       </c>
       <c r="D48" t="s">
-        <v>202</v>
+        <v>247</v>
       </c>
       <c r="E48" t="s">
-        <v>203</v>
+        <v>248</v>
       </c>
       <c r="F48" t="s">
-        <v>204</v>
+        <v>249</v>
       </c>
       <c r="G48">
         <v>1000</v>
@@ -4218,7 +4380,7 @@
         <v>0</v>
       </c>
       <c r="I48" t="s">
-        <v>21</v>
+        <v>250</v>
       </c>
       <c r="J48" t="s">
         <v>22</v>
@@ -4227,13 +4389,13 @@
         <v>22</v>
       </c>
       <c r="L48" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="M48" t="s">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="N48" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="O48">
         <v>1</v>
@@ -4250,16 +4412,16 @@
         <v>16</v>
       </c>
       <c r="C49" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="D49" t="s">
-        <v>206</v>
+        <v>252</v>
       </c>
       <c r="E49" t="s">
-        <v>207</v>
+        <v>253</v>
       </c>
       <c r="F49" t="s">
-        <v>208</v>
+        <v>254</v>
       </c>
       <c r="G49">
         <v>1000</v>
@@ -4268,7 +4430,7 @@
         <v>0</v>
       </c>
       <c r="I49" t="s">
-        <v>21</v>
+        <v>255</v>
       </c>
       <c r="J49" t="s">
         <v>22</v>
@@ -4277,13 +4439,13 @@
         <v>22</v>
       </c>
       <c r="L49" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="M49" t="s">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="N49" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="O49">
         <v>1</v>
@@ -4300,16 +4462,16 @@
         <v>16</v>
       </c>
       <c r="C50" t="s">
-        <v>209</v>
+        <v>256</v>
       </c>
       <c r="D50" t="s">
-        <v>210</v>
+        <v>257</v>
       </c>
       <c r="E50" t="s">
-        <v>211</v>
+        <v>258</v>
       </c>
       <c r="F50" t="s">
-        <v>212</v>
+        <v>259</v>
       </c>
       <c r="G50">
         <v>1000</v>
@@ -4318,7 +4480,7 @@
         <v>0</v>
       </c>
       <c r="I50" t="s">
-        <v>21</v>
+        <v>260</v>
       </c>
       <c r="J50" t="s">
         <v>22</v>
@@ -4327,13 +4489,13 @@
         <v>22</v>
       </c>
       <c r="L50" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="M50" t="s">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="N50" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="O50">
         <v>1</v>
@@ -4350,16 +4512,16 @@
         <v>16</v>
       </c>
       <c r="C51" t="s">
-        <v>213</v>
+        <v>261</v>
       </c>
       <c r="D51" t="s">
-        <v>214</v>
+        <v>262</v>
       </c>
       <c r="E51" t="s">
-        <v>215</v>
+        <v>263</v>
       </c>
       <c r="F51" t="s">
-        <v>216</v>
+        <v>264</v>
       </c>
       <c r="G51">
         <v>1000</v>
@@ -4368,7 +4530,7 @@
         <v>0</v>
       </c>
       <c r="I51" t="s">
-        <v>21</v>
+        <v>265</v>
       </c>
       <c r="J51" t="s">
         <v>22</v>
@@ -4377,18 +4539,68 @@
         <v>22</v>
       </c>
       <c r="L51" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="M51" t="s">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="N51" t="s">
-        <v>199</v>
+        <v>244</v>
       </c>
       <c r="O51">
         <v>1</v>
       </c>
       <c r="P51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16">
+      <c r="A52">
+        <v>1</v>
+      </c>
+      <c r="B52" t="s">
+        <v>16</v>
+      </c>
+      <c r="C52" t="s">
+        <v>266</v>
+      </c>
+      <c r="D52" t="s">
+        <v>267</v>
+      </c>
+      <c r="E52" t="s">
+        <v>268</v>
+      </c>
+      <c r="F52" t="s">
+        <v>269</v>
+      </c>
+      <c r="G52">
+        <v>1000</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52" t="s">
+        <v>270</v>
+      </c>
+      <c r="J52" t="s">
+        <v>22</v>
+      </c>
+      <c r="K52">
+        <v>50</v>
+      </c>
+      <c r="L52" t="s">
+        <v>23</v>
+      </c>
+      <c r="M52" t="s">
+        <v>24</v>
+      </c>
+      <c r="N52">
+        <v>12</v>
+      </c>
+      <c r="O52">
+        <v>1</v>
+      </c>
+      <c r="P52">
         <v>1</v>
       </c>
     </row>

</xml_diff>